<commit_message>
fix: product import field mapping and remove facets from schema
- Fix SEO fields writing to correct path (seo.metaTitle/metaDescription instead of meta.title/description)
- Support Cost Price (CNY) column in Excel import
- Add Weight (kg) and Focus Keyword import support
- Populate categories array with parent category IDs during import
- Remove facets group from Products collection (merged into Specifications)
- Update smart-recommend to extract materials/certifications from specifications
- Update Excel template with new columns (Weight, Focus Keyword, CNY)
- Add listSearchableFields and updatedAt to admin default columns

🤖 Generated with [Qoder][https://qoder.com]
</commit_message>
<xml_diff>
--- a/Machrio_Import_Template_v4.xlsx
+++ b/Machrio_Import_Template_v4.xlsx
@@ -722,7 +722,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -751,6 +751,10 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1163,7 +1167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT3"/>
+  <dimension ref="A1:AV3"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="2"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1178,6 +1182,7 @@
     <col width="13" customWidth="1" min="11" max="12"/>
     <col width="10" customWidth="1" min="13" max="14"/>
     <col width="12" customWidth="1" min="15" max="16"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
     <col width="15" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="17" customWidth="1" min="19" max="19"/>
@@ -1202,6 +1207,7 @@
     <col width="38" customWidth="1" min="38" max="38"/>
     <col width="45" customWidth="1" min="39" max="39"/>
     <col width="32" customWidth="1" min="40" max="40"/>
+    <col width="18" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1257,7 +1263,7 @@
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>Cost Price (USD)</t>
+          <t>Cost Price (CNY)</t>
         </is>
       </c>
       <c r="L1" s="4" t="inlineStr">
@@ -1280,157 +1286,167 @@
           <t>Package Unit</t>
         </is>
       </c>
-      <c r="P1" s="5" t="inlineStr">
+      <c r="P1" s="10" t="inlineStr">
+        <is>
+          <t>Weight (kg)</t>
+        </is>
+      </c>
+      <c r="Q1" s="5" t="inlineStr">
         <is>
           <t>Lead Time</t>
         </is>
       </c>
-      <c r="Q1" s="5" t="inlineStr">
+      <c r="R1" s="5" t="inlineStr">
         <is>
           <t>Availability</t>
         </is>
       </c>
-      <c r="R1" s="5" t="inlineStr">
+      <c r="S1" s="5" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="S1" s="5" t="inlineStr">
+      <c r="T1" s="5" t="inlineStr">
         <is>
           <t>Purchase Mode</t>
         </is>
       </c>
-      <c r="T1" s="6" t="inlineStr">
+      <c r="U1" s="6" t="inlineStr">
         <is>
           <t>Attribute 1 Name</t>
         </is>
       </c>
-      <c r="U1" s="6" t="inlineStr">
+      <c r="V1" s="6" t="inlineStr">
         <is>
           <t>Attribute 1 Value</t>
         </is>
       </c>
-      <c r="V1" s="6" t="inlineStr">
+      <c r="W1" s="6" t="inlineStr">
         <is>
           <t>Attribute 2 Name</t>
         </is>
       </c>
-      <c r="W1" s="6" t="inlineStr">
+      <c r="X1" s="6" t="inlineStr">
         <is>
           <t>Attribute 2 Value</t>
         </is>
       </c>
-      <c r="X1" s="6" t="inlineStr">
+      <c r="Y1" s="6" t="inlineStr">
         <is>
           <t>Attribute 3 Name</t>
         </is>
       </c>
-      <c r="Y1" s="6" t="inlineStr">
+      <c r="Z1" s="6" t="inlineStr">
         <is>
           <t>Attribute 3 Value</t>
         </is>
       </c>
-      <c r="Z1" s="6" t="inlineStr">
+      <c r="AA1" s="6" t="inlineStr">
         <is>
           <t>Attribute 4 Name</t>
         </is>
       </c>
-      <c r="AA1" s="6" t="inlineStr">
+      <c r="AB1" s="6" t="inlineStr">
         <is>
           <t>Attribute 4 Value</t>
         </is>
       </c>
-      <c r="AB1" s="6" t="inlineStr">
+      <c r="AC1" s="6" t="inlineStr">
         <is>
           <t>Attribute 5 Name</t>
         </is>
       </c>
-      <c r="AC1" s="6" t="inlineStr">
+      <c r="AD1" s="6" t="inlineStr">
         <is>
           <t>Attribute 5 Value</t>
         </is>
       </c>
-      <c r="AD1" s="6" t="inlineStr">
+      <c r="AE1" s="6" t="inlineStr">
         <is>
           <t>Attribute 6 Name</t>
         </is>
       </c>
-      <c r="AE1" s="6" t="inlineStr">
+      <c r="AF1" s="6" t="inlineStr">
         <is>
           <t>Attribute 6 Value</t>
         </is>
       </c>
-      <c r="AF1" s="6" t="inlineStr">
+      <c r="AG1" s="6" t="inlineStr">
         <is>
           <t>Attribute 7 Name</t>
         </is>
       </c>
-      <c r="AG1" s="6" t="inlineStr">
+      <c r="AH1" s="6" t="inlineStr">
         <is>
           <t>Attribute 7 Value</t>
         </is>
       </c>
-      <c r="AH1" s="6" t="inlineStr">
+      <c r="AI1" s="6" t="inlineStr">
         <is>
           <t>Attribute 8 Name</t>
         </is>
       </c>
-      <c r="AI1" s="6" t="inlineStr">
+      <c r="AJ1" s="6" t="inlineStr">
         <is>
           <t>Attribute 8 Value</t>
         </is>
       </c>
-      <c r="AJ1" s="6" t="inlineStr">
+      <c r="AK1" s="6" t="inlineStr">
         <is>
           <t>Attribute 9 Name</t>
         </is>
       </c>
-      <c r="AK1" s="6" t="inlineStr">
+      <c r="AL1" s="6" t="inlineStr">
         <is>
           <t>Attribute 9 Value</t>
         </is>
       </c>
-      <c r="AL1" s="7" t="inlineStr">
+      <c r="AM1" s="7" t="inlineStr">
         <is>
           <t>Meta Title</t>
         </is>
       </c>
-      <c r="AM1" s="7" t="inlineStr">
+      <c r="AN1" s="7" t="inlineStr">
         <is>
           <t>Meta Description</t>
         </is>
       </c>
-      <c r="AN1" s="7" t="inlineStr">
+      <c r="AO1" s="10" t="inlineStr">
+        <is>
+          <t>Focus Keyword</t>
+        </is>
+      </c>
+      <c r="AP1" s="7" t="inlineStr">
         <is>
           <t>Source URL</t>
         </is>
       </c>
-      <c r="AO1" s="7" t="inlineStr">
+      <c r="AQ1" s="7" t="inlineStr">
         <is>
           <t>FAQ Question 1</t>
         </is>
       </c>
-      <c r="AP1" s="7" t="inlineStr">
+      <c r="AR1" s="7" t="inlineStr">
         <is>
           <t>FAQ Answer 1</t>
         </is>
       </c>
-      <c r="AQ1" s="7" t="inlineStr">
+      <c r="AS1" s="7" t="inlineStr">
         <is>
           <t>FAQ Question 2</t>
         </is>
       </c>
-      <c r="AR1" s="7" t="inlineStr">
+      <c r="AT1" s="7" t="inlineStr">
         <is>
           <t>FAQ Answer 2</t>
         </is>
       </c>
-      <c r="AS1" s="7" t="inlineStr">
+      <c r="AU1" s="7" t="inlineStr">
         <is>
           <t>FAQ Question 3</t>
         </is>
       </c>
-      <c r="AT1" s="7" t="inlineStr">
+      <c r="AV1" s="7" t="inlineStr">
         <is>
           <t>FAQ Answer 3</t>
         </is>
@@ -1489,7 +1505,7 @@
       </c>
       <c r="K2" s="8" t="inlineStr">
         <is>
-          <t>Cost in USD</t>
+          <t>Cost in CNY</t>
         </is>
       </c>
       <c r="L2" s="8" t="inlineStr">
@@ -1512,157 +1528,167 @@
           <t>Each/Pair/Box</t>
         </is>
       </c>
-      <c r="P2" s="8" t="inlineStr">
+      <c r="P2" s="11" t="inlineStr">
+        <is>
+          <t>Weight in kg</t>
+        </is>
+      </c>
+      <c r="Q2" s="8" t="inlineStr">
         <is>
           <t>2-3 weeks</t>
         </is>
       </c>
-      <c r="Q2" s="8" t="inlineStr">
+      <c r="R2" s="8" t="inlineStr">
         <is>
           <t>In Stock / Made to Order</t>
         </is>
       </c>
-      <c r="R2" s="8" t="inlineStr">
+      <c r="S2" s="8" t="inlineStr">
         <is>
           <t>Draft / Active</t>
         </is>
       </c>
-      <c r="S2" s="8" t="inlineStr">
+      <c r="T2" s="8" t="inlineStr">
         <is>
           <t>Buy Online + RFQ</t>
         </is>
       </c>
-      <c r="T2" s="8" t="inlineStr">
+      <c r="U2" s="8" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="U2" s="8" t="inlineStr">
+      <c r="V2" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="V2" s="8" t="inlineStr">
+      <c r="W2" s="8" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="W2" s="8" t="inlineStr">
+      <c r="X2" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="X2" s="8" t="inlineStr">
+      <c r="Y2" s="8" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="Y2" s="8" t="inlineStr">
+      <c r="Z2" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="Z2" s="8" t="inlineStr">
+      <c r="AA2" s="8" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="AA2" s="8" t="inlineStr">
+      <c r="AB2" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="AB2" s="8" t="inlineStr">
+      <c r="AC2" s="8" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="AC2" s="8" t="inlineStr">
+      <c r="AD2" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="AD2" s="8" t="inlineStr">
+      <c r="AE2" s="8" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="AE2" s="8" t="inlineStr">
+      <c r="AF2" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="AF2" s="8" t="inlineStr">
+      <c r="AG2" s="8" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="AG2" s="8" t="inlineStr">
+      <c r="AH2" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="AH2" s="8" t="inlineStr">
+      <c r="AI2" s="8" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="AI2" s="8" t="inlineStr">
+      <c r="AJ2" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="AJ2" s="8" t="inlineStr">
+      <c r="AK2" s="8" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="AK2" s="8" t="inlineStr">
+      <c r="AL2" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="AL2" s="8" t="inlineStr">
+      <c r="AM2" s="8" t="inlineStr">
         <is>
           <t>Max 70 chars | Machrio</t>
         </is>
       </c>
-      <c r="AM2" s="8" t="inlineStr">
+      <c r="AN2" s="8" t="inlineStr">
         <is>
           <t>Max 160 chars</t>
         </is>
       </c>
-      <c r="AN2" s="8" t="inlineStr">
+      <c r="AO2" s="11" t="inlineStr">
+        <is>
+          <t>Primary keyword</t>
+        </is>
+      </c>
+      <c r="AP2" s="8" t="inlineStr">
         <is>
           <t>Original URL</t>
         </is>
       </c>
-      <c r="AO2" s="8" t="inlineStr">
+      <c r="AQ2" s="8" t="inlineStr">
         <is>
           <t>Question text</t>
         </is>
       </c>
-      <c r="AP2" s="8" t="inlineStr">
+      <c r="AR2" s="8" t="inlineStr">
         <is>
           <t>Answer text</t>
         </is>
       </c>
-      <c r="AQ2" s="8" t="inlineStr">
+      <c r="AS2" s="8" t="inlineStr">
         <is>
           <t>Question text</t>
         </is>
       </c>
-      <c r="AR2" s="8" t="inlineStr">
+      <c r="AT2" s="8" t="inlineStr">
         <is>
           <t>Answer text</t>
         </is>
       </c>
-      <c r="AS2" s="8" t="inlineStr">
+      <c r="AU2" s="8" t="inlineStr">
         <is>
           <t>Question text</t>
         </is>
       </c>
-      <c r="AT2" s="8" t="inlineStr">
+      <c r="AV2" s="8" t="inlineStr">
         <is>
           <t>Answer text</t>
         </is>
@@ -1740,129 +1766,123 @@
           <t>Pair</t>
         </is>
       </c>
-      <c r="P3" s="9" t="inlineStr">
+      <c r="Q3" s="9" t="inlineStr">
         <is>
           <t>2-3 weeks</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
+      <c r="R3" s="9" t="inlineStr">
         <is>
           <t>In Stock</t>
         </is>
       </c>
-      <c r="R3" s="9" t="inlineStr">
+      <c r="S3" s="9" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S3" s="9" t="inlineStr">
+      <c r="T3" s="9" t="inlineStr">
         <is>
           <t>Buy Online + RFQ</t>
         </is>
       </c>
-      <c r="T3" s="9" t="inlineStr">
+      <c r="U3" s="9" t="inlineStr">
         <is>
           <t>Size</t>
         </is>
       </c>
-      <c r="U3" s="9" t="inlineStr">
+      <c r="V3" s="9" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="V3" s="9" t="inlineStr">
+      <c r="W3" s="9" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="W3" s="9" t="inlineStr">
+      <c r="X3" s="9" t="inlineStr">
         <is>
           <t>HPPE Blend</t>
         </is>
       </c>
-      <c r="X3" s="9" t="inlineStr">
+      <c r="Y3" s="9" t="inlineStr">
         <is>
           <t>Standards</t>
         </is>
       </c>
-      <c r="Y3" s="9" t="inlineStr">
+      <c r="Z3" s="9" t="inlineStr">
         <is>
           <t>EN 388:2016</t>
         </is>
       </c>
-      <c r="Z3" s="9" t="inlineStr">
+      <c r="AA3" s="9" t="inlineStr">
         <is>
           <t>ANSI Rating</t>
         </is>
       </c>
-      <c r="AA3" s="9" t="inlineStr">
+      <c r="AB3" s="9" t="inlineStr">
         <is>
           <t>A4</t>
         </is>
       </c>
-      <c r="AB3" s="9" t="inlineStr">
+      <c r="AC3" s="9" t="inlineStr">
         <is>
           <t>Glove Size</t>
         </is>
       </c>
-      <c r="AC3" s="9" t="inlineStr">
+      <c r="AD3" s="9" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="AD3" s="9" t="inlineStr">
+      <c r="AE3" s="9" t="inlineStr">
         <is>
           <t>Glove Material</t>
         </is>
       </c>
-      <c r="AE3" s="9" t="inlineStr">
+      <c r="AF3" s="9" t="inlineStr">
         <is>
           <t>HPPE</t>
         </is>
       </c>
-      <c r="AF3" s="9" t="inlineStr">
+      <c r="AG3" s="9" t="inlineStr">
         <is>
           <t>Cut Level</t>
         </is>
       </c>
-      <c r="AG3" s="9" t="inlineStr">
+      <c r="AH3" s="9" t="inlineStr">
         <is>
           <t>A4</t>
         </is>
       </c>
-      <c r="AH3" s="9" t="inlineStr">
+      <c r="AI3" s="9" t="inlineStr">
         <is>
           <t>Coating</t>
         </is>
       </c>
-      <c r="AI3" s="9" t="inlineStr">
+      <c r="AJ3" s="9" t="inlineStr">
         <is>
           <t>Nitrile</t>
         </is>
       </c>
-      <c r="AJ3" s="9" t="inlineStr"/>
       <c r="AK3" s="9" t="inlineStr"/>
-      <c r="AL3" s="9" t="inlineStr">
+      <c r="AL3" s="9" t="inlineStr"/>
+      <c r="AM3" s="9" t="inlineStr">
         <is>
           <t>Cut Resistant Gloves Size 9 | Machrio</t>
         </is>
       </c>
-      <c r="AM3" s="9" t="inlineStr">
+      <c r="AN3" s="9" t="inlineStr">
         <is>
           <t>Buy Safety Gloves at competitive prices. ANSI A4 rated.</t>
         </is>
       </c>
-      <c r="AN3" s="9" t="inlineStr">
+      <c r="AP3" s="9" t="inlineStr">
         <is>
           <t>https://www.zkh.com/item/HP4853.html</t>
         </is>
       </c>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AN3"/>

</xml_diff>